<commit_message>
added some dataanalysis to be removed at the end
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4E7FB2-1CAC-4FA4-91DD-590DC3CE59E3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B36FFC-F06F-4FD0-9CAE-5B4BD3B9BA46}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="hydrogen-transport" sheetId="1" r:id="rId1"/>
     <sheet name="Parameters" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
@@ -858,7 +858,7 @@
   <dimension ref="A1:R49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" customWidth="1"/>
+    <col min="1" max="1" width="55.88671875" customWidth="1"/>
     <col min="3" max="3" width="16.44140625" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
     <col min="5" max="5" width="13.77734375" customWidth="1"/>

</xml_diff>

<commit_message>
Implementing dataanalysis of xarray containing mapped variables
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B36FFC-F06F-4FD0-9CAE-5B4BD3B9BA46}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7EFCA8-115B-465F-B417-9FB7AD3D37A7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -859,7 +859,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="55.88671875" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" customWidth="1"/>
+    <col min="3" max="3" width="33.21875" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
     <col min="5" max="5" width="13.77734375" customWidth="1"/>
     <col min="6" max="6" width="17.109375" customWidth="1"/>

</xml_diff>

<commit_message>
assign transport activities according to the decision tree
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD434366-C89D-4D33-A3BE-D509CC2B5F6D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C8414FC-1405-4F9C-8A66-41FC458B3A88}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="hydrogen-transport" sheetId="1" r:id="rId1"/>
-    <sheet name="ship" sheetId="3" r:id="rId2"/>
-    <sheet name="Parameters" sheetId="2" r:id="rId3"/>
+    <sheet name="hydrogen-transport (2)" sheetId="4" r:id="rId2"/>
+    <sheet name="ship" sheetId="3" r:id="rId3"/>
+    <sheet name="Parameters" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="169">
   <si>
     <t>Database</t>
   </si>
@@ -472,33 +473,6 @@
     <t>C. Wulf et al. / Journal of Cleaner Production 199 (2018) 431-443</t>
   </si>
   <si>
-    <t>Car db</t>
-  </si>
-  <si>
-    <t>ecoinvent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">transport, gaseous hydrogen, lorry </t>
-  </si>
-  <si>
-    <t>market for hydrogen</t>
-  </si>
-  <si>
-    <t>hydrogen, gaseous</t>
-  </si>
-  <si>
-    <t>market for electricity</t>
-  </si>
-  <si>
-    <t>transport, gaseous hydrogen, lorry, market average propulsion system</t>
-  </si>
-  <si>
-    <t>transport, liquid hydrogen, lorry, market average propulsion system</t>
-  </si>
-  <si>
-    <t xml:space="preserve">transport, liquid hydrogen, lorry </t>
-  </si>
-  <si>
     <t>LCI for gaseous hydrogen transport for 1 tkm. Storage tank taken from the hydrogen-distribution dataset. Lorry is market average. Boil-off losses are 0.5 % and 0.5 % during compression (Reuß et al. 2019)</t>
   </si>
   <si>
@@ -508,9 +482,6 @@
     <t>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</t>
   </si>
   <si>
-    <t>kWh</t>
-  </si>
-  <si>
     <t>electricity, medium voltage</t>
   </si>
   <si>
@@ -539,6 +510,45 @@
   </si>
   <si>
     <t>air</t>
+  </si>
+  <si>
+    <t>market for hydrogen, gaseous, low pressure</t>
+  </si>
+  <si>
+    <t>hydrogen, gaseous, low pressure</t>
+  </si>
+  <si>
+    <t>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</t>
+  </si>
+  <si>
+    <t>transport, hydrogen, gaseous, lorry, market average propulsion system</t>
+  </si>
+  <si>
+    <t>this dataset is used as a proxy</t>
+  </si>
+  <si>
+    <t>market for electricity, medium voltage</t>
+  </si>
+  <si>
+    <t>LCI for hydrogen transport as liquid ammonia for 1 tkm. Storage tank taken from the hydrogen-distribution dataset. Market average. Boil-off losses are 3 % and 1.65 % during liquefaction (Reuß et al. 2019)</t>
+  </si>
+  <si>
+    <t>LCI for liquid hydrogen transport for 1 tkm. Storage tank taken from the hydrogen-distribution dataset. Ship is market average. Boil-off losses are 3 % and 1.65 % during liquefaction (Reuß et al. 2019)</t>
+  </si>
+  <si>
+    <t>kilowatt hour</t>
+  </si>
+  <si>
+    <t>RER</t>
+  </si>
+  <si>
+    <t>transport, hydrogen, gaseous, lorry , market average propulsion system</t>
+  </si>
+  <si>
+    <t>transport, hydrogen, liquid, lorry, market average propulsion system</t>
+  </si>
+  <si>
+    <t>DE</t>
   </si>
 </sst>
 </file>
@@ -943,663 +953,821 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="82.6640625" customWidth="1"/>
-    <col min="3" max="3" width="33.21875" customWidth="1"/>
-    <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="13.77734375" customWidth="1"/>
-    <col min="6" max="6" width="17.109375" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="7" max="7" width="85.44140625" customWidth="1"/>
     <col min="8" max="8" width="25.44140625" customWidth="1"/>
-    <col min="12" max="12" width="13.21875" customWidth="1"/>
-    <col min="13" max="13" width="43.88671875" customWidth="1"/>
-    <col min="14" max="14" width="13.33203125" customWidth="1"/>
-    <col min="15" max="15" width="14.33203125" customWidth="1"/>
+    <col min="11" max="11" width="13.21875" customWidth="1"/>
+    <col min="12" max="12" width="43.88671875" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B1" s="3" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B3" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="str">
+        <f>B6</f>
+        <v>transport, hydrogen, gaseous, lorry, market average propulsion system</v>
+      </c>
+      <c r="B12">
+        <f>B5</f>
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" t="str">
+        <f>A12</f>
+        <v>transport, hydrogen, gaseous, lorry, market average propulsion system</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" t="s">
+        <v>151</v>
+      </c>
+      <c r="I13" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>140</v>
+      </c>
+      <c r="B14">
+        <f>1*1000</f>
+        <v>1000</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" t="s">
+        <v>140</v>
+      </c>
+      <c r="I14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B15">
+        <f>1000*0.005</f>
+        <v>5</v>
+      </c>
+      <c r="C15" t="s">
+        <v>165</v>
+      </c>
+      <c r="D15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" t="s">
+        <v>157</v>
+      </c>
+      <c r="I15" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>152</v>
+      </c>
+      <c r="B16">
+        <f>1000*0.005</f>
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" t="s">
+        <v>155</v>
+      </c>
+      <c r="F16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>7</v>
       </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>141</v>
       </c>
-      <c r="B6">
+      <c r="B20">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>15</v>
       </c>
-      <c r="B7" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B21" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B22" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>6</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>11</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" t="s">
+        <v>20</v>
+      </c>
+      <c r="I26" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" t="str">
+        <f>B21</f>
+        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
+      </c>
+      <c r="B27">
+        <f>B20</f>
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" t="s">
+        <v>17</v>
+      </c>
+      <c r="G27" t="str">
+        <f>A27</f>
+        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>140</v>
+      </c>
+      <c r="B28">
+        <v>1000</v>
+      </c>
+      <c r="C28" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" t="s">
+        <v>26</v>
+      </c>
+      <c r="F28" t="s">
+        <v>18</v>
+      </c>
+      <c r="G28" t="s">
+        <v>140</v>
+      </c>
+      <c r="I28" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B29">
+        <f>1000*0.01625</f>
+        <v>16.25</v>
+      </c>
+      <c r="C29" t="s">
+        <v>165</v>
+      </c>
+      <c r="D29" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" t="s">
+        <v>157</v>
+      </c>
+      <c r="I29" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>161</v>
+      </c>
+      <c r="B30">
+        <f>1000*6.78</f>
+        <v>6780</v>
+      </c>
+      <c r="C30" t="s">
+        <v>168</v>
+      </c>
+      <c r="D30" t="s">
+        <v>164</v>
+      </c>
+      <c r="F30" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30" t="s">
+        <v>146</v>
+      </c>
+      <c r="I30" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>161</v>
+      </c>
+      <c r="B31">
+        <v>0.6</v>
+      </c>
+      <c r="C31" t="s">
+        <v>168</v>
+      </c>
+      <c r="D31" t="s">
+        <v>164</v>
+      </c>
+      <c r="F31" t="s">
+        <v>18</v>
+      </c>
+      <c r="G31" t="s">
+        <v>146</v>
+      </c>
+      <c r="I31" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F12" t="s">
-        <v>23</v>
-      </c>
-      <c r="G12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H12" t="s">
-        <v>20</v>
-      </c>
-      <c r="I12" t="s">
-        <v>15</v>
-      </c>
-      <c r="J12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" t="str">
-        <f>B7</f>
-        <v xml:space="preserve">transport, gaseous hydrogen, lorry </v>
-      </c>
-      <c r="B13">
-        <f>B6</f>
-        <v>1</v>
-      </c>
-      <c r="C13" t="str">
-        <f>B2</f>
-        <v>hydrogen-transport</v>
-      </c>
-      <c r="D13" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" t="s">
-        <v>16</v>
-      </c>
-      <c r="G13" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>160</v>
-      </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
-      <c r="C14" t="s">
-        <v>144</v>
-      </c>
-      <c r="D14" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G14" t="s">
-        <v>18</v>
-      </c>
-      <c r="I14" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>140</v>
-      </c>
-      <c r="B15">
-        <v>1200</v>
-      </c>
-      <c r="C15" t="s">
-        <v>144</v>
-      </c>
-      <c r="D15" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="B32">
+        <f>1000*0.01625</f>
+        <v>16.25</v>
+      </c>
+      <c r="D32" t="s">
         <v>26</v>
-      </c>
-      <c r="G15" t="s">
-        <v>18</v>
-      </c>
-      <c r="I15" t="s">
-        <v>140</v>
-      </c>
-      <c r="J15" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="B16">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C16" t="s">
-        <v>144</v>
-      </c>
-      <c r="D16" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" t="s">
-        <v>26</v>
-      </c>
-      <c r="G16" t="s">
-        <v>18</v>
-      </c>
-      <c r="I16" t="s">
-        <v>147</v>
-      </c>
-      <c r="J16" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>162</v>
-      </c>
-      <c r="B17">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C17" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17" t="s">
-        <v>26</v>
-      </c>
-      <c r="F17" t="s">
-        <v>165</v>
-      </c>
-      <c r="G17" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>141</v>
-      </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>14</v>
-      </c>
-      <c r="B23" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>6</v>
-      </c>
-      <c r="B25" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" t="s">
-        <v>12</v>
-      </c>
-      <c r="C27" t="s">
-        <v>13</v>
-      </c>
-      <c r="D27" t="s">
-        <v>7</v>
-      </c>
-      <c r="E27" t="s">
-        <v>14</v>
-      </c>
-      <c r="F27" t="s">
-        <v>23</v>
-      </c>
-      <c r="G27" t="s">
-        <v>9</v>
-      </c>
-      <c r="H27" t="s">
-        <v>20</v>
-      </c>
-      <c r="I27" t="s">
-        <v>15</v>
-      </c>
-      <c r="J27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A28" t="str">
-        <f>B22</f>
-        <v xml:space="preserve">transport, liquid hydrogen, lorry </v>
-      </c>
-      <c r="B28">
-        <f>B21</f>
-        <v>1</v>
-      </c>
-      <c r="C28" t="str">
-        <f>B2</f>
-        <v>hydrogen-transport</v>
-      </c>
-      <c r="D28" t="s">
-        <v>8</v>
-      </c>
-      <c r="E28" t="s">
-        <v>16</v>
-      </c>
-      <c r="G28" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>140</v>
-      </c>
-      <c r="B29">
-        <v>4300</v>
-      </c>
-      <c r="C29" t="s">
-        <v>144</v>
-      </c>
-      <c r="D29" t="s">
-        <v>8</v>
-      </c>
-      <c r="E29" t="s">
-        <v>26</v>
-      </c>
-      <c r="G29" t="s">
-        <v>18</v>
-      </c>
-      <c r="I29" t="s">
-        <v>140</v>
-      </c>
-      <c r="J29" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="B30">
-        <v>1.6250000000000001E-2</v>
-      </c>
-      <c r="C30" t="s">
-        <v>144</v>
-      </c>
-      <c r="D30" t="s">
-        <v>8</v>
-      </c>
-      <c r="E30" t="s">
-        <v>26</v>
-      </c>
-      <c r="G30" t="s">
-        <v>18</v>
-      </c>
-      <c r="I30" t="s">
-        <v>147</v>
-      </c>
-      <c r="J30" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>148</v>
-      </c>
-      <c r="B31">
-        <v>6.78</v>
-      </c>
-      <c r="C31" t="s">
-        <v>144</v>
-      </c>
-      <c r="D31" t="s">
-        <v>8</v>
-      </c>
-      <c r="E31" t="s">
-        <v>155</v>
-      </c>
-      <c r="G31" t="s">
-        <v>18</v>
-      </c>
-      <c r="I31" t="s">
-        <v>156</v>
-      </c>
-      <c r="J31" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>148</v>
-      </c>
-      <c r="B32">
-        <v>0.6</v>
-      </c>
-      <c r="C32" t="s">
-        <v>144</v>
-      </c>
-      <c r="D32" t="s">
-        <v>8</v>
       </c>
       <c r="E32" t="s">
         <v>155</v>
       </c>
-      <c r="G32" t="s">
-        <v>18</v>
-      </c>
-      <c r="I32" t="s">
-        <v>156</v>
-      </c>
-      <c r="J32" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>162</v>
-      </c>
-      <c r="B33">
-        <v>1.6250000000000001E-2</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="F32" t="s">
         <v>27</v>
       </c>
-      <c r="E33" t="s">
-        <v>26</v>
-      </c>
-      <c r="F33" t="s">
-        <v>165</v>
-      </c>
-      <c r="G33" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
+    </row>
+    <row r="34" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B34" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>141</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>15</v>
+      </c>
+      <c r="B37" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>14</v>
+      </c>
+      <c r="B38" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>6</v>
+      </c>
+      <c r="B40" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>11</v>
+      </c>
+      <c r="B42" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" t="s">
         <v>7</v>
       </c>
-      <c r="B36" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>141</v>
-      </c>
-      <c r="B37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
+      <c r="D42" t="s">
+        <v>14</v>
+      </c>
+      <c r="E42" t="s">
+        <v>23</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+      <c r="G42" t="s">
         <v>15</v>
-      </c>
-      <c r="B38" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>14</v>
-      </c>
-      <c r="B39" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>6</v>
-      </c>
-      <c r="B41" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="H42" t="s">
         <v>20</v>
       </c>
       <c r="I42" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" t="str">
+        <f>B37</f>
+        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
+      </c>
+      <c r="B43">
+        <f>B36</f>
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
+        <v>8</v>
+      </c>
+      <c r="D43" t="s">
+        <v>16</v>
+      </c>
+      <c r="F43" t="s">
+        <v>17</v>
+      </c>
+      <c r="G43" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>140</v>
+      </c>
+      <c r="B44">
+        <f>1000*1</f>
+        <v>1000</v>
+      </c>
+      <c r="C44" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" t="s">
+        <v>26</v>
+      </c>
+      <c r="F44" t="s">
+        <v>18</v>
+      </c>
+      <c r="G44" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B45">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C45" t="s">
+        <v>165</v>
+      </c>
+      <c r="D45" t="s">
+        <v>26</v>
+      </c>
+      <c r="F45" t="s">
+        <v>18</v>
+      </c>
+      <c r="G45" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>153</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" t="s">
+        <v>16</v>
+      </c>
+      <c r="F46" t="s">
+        <v>18</v>
+      </c>
+      <c r="G46" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>7</v>
+      </c>
+      <c r="B49" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>141</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
         <v>15</v>
       </c>
-      <c r="J42" t="s">
+      <c r="B51" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>14</v>
+      </c>
+      <c r="B52" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
+      <c r="B54" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
         <v>11</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B56" t="s">
         <v>12</v>
       </c>
-      <c r="C43" t="s">
-        <v>13</v>
-      </c>
-      <c r="D43" t="s">
+      <c r="C56" t="s">
         <v>7</v>
       </c>
-      <c r="E43" t="s">
+      <c r="D56" t="s">
         <v>14</v>
       </c>
-      <c r="F43" t="s">
+      <c r="E56" t="s">
         <v>23</v>
       </c>
-      <c r="G43" t="s">
+      <c r="F56" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A44" t="str">
-        <f>B38</f>
-        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
-      </c>
-      <c r="B44">
-        <f>B37</f>
+      <c r="G56" t="s">
+        <v>15</v>
+      </c>
+      <c r="H56" t="s">
+        <v>20</v>
+      </c>
+      <c r="I56" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A57" t="str">
+        <f>B51</f>
+        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
+      </c>
+      <c r="B57">
+        <f>B50</f>
         <v>1</v>
       </c>
-      <c r="C44" t="str">
-        <f>B2</f>
-        <v>hydrogen-transport</v>
-      </c>
-      <c r="D44" t="s">
-        <v>8</v>
-      </c>
-      <c r="E44" t="s">
+      <c r="C57" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57" t="s">
         <v>16</v>
       </c>
-      <c r="G44" t="s">
+      <c r="F57" t="s">
         <v>17</v>
       </c>
-      <c r="I44" t="s">
+      <c r="G57" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>140</v>
+      </c>
+      <c r="B58">
+        <v>0</v>
+      </c>
+      <c r="C58" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58" t="s">
+        <v>26</v>
+      </c>
+      <c r="F58" t="s">
+        <v>18</v>
+      </c>
+      <c r="G58" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A59" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B59">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>165</v>
+      </c>
+      <c r="D59" t="s">
+        <v>26</v>
+      </c>
+      <c r="F59" t="s">
+        <v>18</v>
+      </c>
+      <c r="G59" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>153</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>8</v>
+      </c>
+      <c r="D60" t="s">
+        <v>16</v>
+      </c>
+      <c r="F60" t="s">
+        <v>18</v>
+      </c>
+      <c r="G60" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>140</v>
-      </c>
-      <c r="B45">
-        <v>1</v>
-      </c>
-      <c r="C45" t="s">
-        <v>143</v>
-      </c>
-      <c r="D45" t="s">
-        <v>8</v>
-      </c>
-      <c r="E45" t="s">
-        <v>26</v>
-      </c>
-      <c r="G45" t="s">
-        <v>18</v>
-      </c>
-      <c r="I45" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="B46">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C46" t="s">
-        <v>144</v>
-      </c>
-      <c r="D46" t="s">
-        <v>8</v>
-      </c>
-      <c r="E46" t="s">
-        <v>26</v>
-      </c>
-      <c r="G46" t="s">
-        <v>18</v>
-      </c>
-      <c r="I46" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>163</v>
-      </c>
-      <c r="B47">
-        <v>1</v>
-      </c>
-      <c r="C47" t="s">
-        <v>144</v>
-      </c>
-      <c r="D47" t="s">
-        <v>8</v>
-      </c>
-      <c r="E47" t="s">
-        <v>26</v>
-      </c>
-      <c r="G47" t="s">
-        <v>18</v>
-      </c>
-      <c r="I47" t="s">
-        <v>164</v>
-      </c>
+    <row r="62" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A62" s="1"/>
+      <c r="B62" s="1"/>
+    </row>
+    <row r="69" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A69" s="1"/>
+    </row>
+    <row r="72" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A72" s="4"/>
+    </row>
+    <row r="73" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A73" s="4"/>
+    </row>
+    <row r="74" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A74" s="4"/>
+    </row>
+    <row r="75" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A75" s="4"/>
+      <c r="G75" s="4"/>
+    </row>
+    <row r="77" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A77" s="4"/>
+    </row>
+    <row r="78" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A78" s="4"/>
+    </row>
+    <row r="79" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A79" s="4"/>
+    </row>
+    <row r="80" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A80" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1608,392 +1776,1179 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFCFE87B-D030-4AA0-99E6-3DBA7D6E9B67}">
+  <dimension ref="A1:I81"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="82.6640625" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="7" max="7" width="85.44140625" customWidth="1"/>
+    <col min="8" max="8" width="25.44140625" customWidth="1"/>
+    <col min="11" max="11" width="13.21875" customWidth="1"/>
+    <col min="12" max="12" width="43.88671875" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
+        <v>20</v>
+      </c>
+      <c r="I12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="str">
+        <f>B7</f>
+        <v>transport, hydrogen, gaseous, lorry , market average propulsion system</v>
+      </c>
+      <c r="B13">
+        <f>B6</f>
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" t="str">
+        <f>A13</f>
+        <v>transport, hydrogen, gaseous, lorry , market average propulsion system</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>150</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" t="s">
+        <v>151</v>
+      </c>
+      <c r="I14" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>140</v>
+      </c>
+      <c r="B15">
+        <f>1*1000</f>
+        <v>1000</v>
+      </c>
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" t="s">
+        <v>140</v>
+      </c>
+      <c r="I15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B16">
+        <f>1000*0.005</f>
+        <v>5</v>
+      </c>
+      <c r="C16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" t="s">
+        <v>157</v>
+      </c>
+      <c r="I16" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>152</v>
+      </c>
+      <c r="B17">
+        <f>1000*0.005</f>
+        <v>5</v>
+      </c>
+      <c r="D17" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" t="s">
+        <v>155</v>
+      </c>
+      <c r="F17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>141</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" t="s">
+        <v>20</v>
+      </c>
+      <c r="I27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" t="str">
+        <f>B22</f>
+        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
+      </c>
+      <c r="B28">
+        <f>B21</f>
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" t="s">
+        <v>17</v>
+      </c>
+      <c r="G28" t="str">
+        <f>A28</f>
+        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>140</v>
+      </c>
+      <c r="B29">
+        <v>1000</v>
+      </c>
+      <c r="C29" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" t="s">
+        <v>140</v>
+      </c>
+      <c r="I29" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B30">
+        <f>1000*0.01625</f>
+        <v>16.25</v>
+      </c>
+      <c r="C30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30" t="s">
+        <v>157</v>
+      </c>
+      <c r="I30" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>161</v>
+      </c>
+      <c r="B31">
+        <f>1000*6.78</f>
+        <v>6780</v>
+      </c>
+      <c r="C31" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" t="s">
+        <v>164</v>
+      </c>
+      <c r="F31" t="s">
+        <v>18</v>
+      </c>
+      <c r="G31" t="s">
+        <v>146</v>
+      </c>
+      <c r="I31" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>161</v>
+      </c>
+      <c r="B32">
+        <v>0.6</v>
+      </c>
+      <c r="C32" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" t="s">
+        <v>164</v>
+      </c>
+      <c r="F32" t="s">
+        <v>18</v>
+      </c>
+      <c r="G32" t="s">
+        <v>146</v>
+      </c>
+      <c r="I32" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>152</v>
+      </c>
+      <c r="B33">
+        <f>1000*0.01625</f>
+        <v>16.25</v>
+      </c>
+      <c r="D33" t="s">
+        <v>26</v>
+      </c>
+      <c r="E33" t="s">
+        <v>155</v>
+      </c>
+      <c r="F33" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>141</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>15</v>
+      </c>
+      <c r="B38" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>14</v>
+      </c>
+      <c r="B39" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>6</v>
+      </c>
+      <c r="B41" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>11</v>
+      </c>
+      <c r="B43" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" t="s">
+        <v>7</v>
+      </c>
+      <c r="D43" t="s">
+        <v>14</v>
+      </c>
+      <c r="E43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+      <c r="G43" t="s">
+        <v>15</v>
+      </c>
+      <c r="H43" t="s">
+        <v>20</v>
+      </c>
+      <c r="I43" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" t="str">
+        <f>B38</f>
+        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
+      </c>
+      <c r="B44">
+        <f>B37</f>
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" t="s">
+        <v>16</v>
+      </c>
+      <c r="F44" t="s">
+        <v>17</v>
+      </c>
+      <c r="G44" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>140</v>
+      </c>
+      <c r="B45">
+        <f>1000*1</f>
+        <v>1000</v>
+      </c>
+      <c r="C45" t="s">
+        <v>8</v>
+      </c>
+      <c r="D45" t="s">
+        <v>26</v>
+      </c>
+      <c r="F45" t="s">
+        <v>18</v>
+      </c>
+      <c r="G45" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B46">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" t="s">
+        <v>26</v>
+      </c>
+      <c r="F46" t="s">
+        <v>18</v>
+      </c>
+      <c r="G46" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>153</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" t="s">
+        <v>16</v>
+      </c>
+      <c r="F47" t="s">
+        <v>18</v>
+      </c>
+      <c r="G47" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>7</v>
+      </c>
+      <c r="B50" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>141</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>15</v>
+      </c>
+      <c r="B52" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>14</v>
+      </c>
+      <c r="B53" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>6</v>
+      </c>
+      <c r="B55" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>11</v>
+      </c>
+      <c r="B57" t="s">
+        <v>12</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57" t="s">
+        <v>14</v>
+      </c>
+      <c r="E57" t="s">
+        <v>23</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+      <c r="G57" t="s">
+        <v>15</v>
+      </c>
+      <c r="H57" t="s">
+        <v>20</v>
+      </c>
+      <c r="I57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A58" t="str">
+        <f>B52</f>
+        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
+      </c>
+      <c r="B58">
+        <f>B51</f>
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58" t="s">
+        <v>16</v>
+      </c>
+      <c r="F58" t="s">
+        <v>17</v>
+      </c>
+      <c r="G58" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>140</v>
+      </c>
+      <c r="B59">
+        <v>0</v>
+      </c>
+      <c r="C59" t="s">
+        <v>8</v>
+      </c>
+      <c r="D59" t="s">
+        <v>26</v>
+      </c>
+      <c r="F59" t="s">
+        <v>18</v>
+      </c>
+      <c r="G59" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A60" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B60">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C60" t="s">
+        <v>8</v>
+      </c>
+      <c r="D60" t="s">
+        <v>26</v>
+      </c>
+      <c r="F60" t="s">
+        <v>18</v>
+      </c>
+      <c r="G60" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>153</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61" t="s">
+        <v>16</v>
+      </c>
+      <c r="F61" t="s">
+        <v>18</v>
+      </c>
+      <c r="G61" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A63" s="1"/>
+      <c r="B63" s="1"/>
+    </row>
+    <row r="70" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A70" s="1"/>
+    </row>
+    <row r="73" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A73" s="4"/>
+    </row>
+    <row r="74" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A74" s="4"/>
+    </row>
+    <row r="75" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A75" s="4"/>
+    </row>
+    <row r="76" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A76" s="4"/>
+      <c r="G76" s="4"/>
+    </row>
+    <row r="78" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A78" s="4"/>
+    </row>
+    <row r="79" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A79" s="4"/>
+    </row>
+    <row r="80" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A80" s="4"/>
+    </row>
+    <row r="81" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A81" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AF05BD3-82B5-4829-9975-BAE4BAEB41CD}">
-  <dimension ref="A1:R49"/>
+  <dimension ref="A1:R50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.5546875" customWidth="1"/>
+    <col min="3" max="3" width="19.21875" customWidth="1"/>
+    <col min="8" max="8" width="26.33203125" customWidth="1"/>
+    <col min="15" max="15" width="27.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B2" s="3" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1"/>
-      <c r="B2" s="3"/>
-    </row>
     <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
+    </row>
+    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="8" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>126</v>
-      </c>
-      <c r="B8" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>126</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>136</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>14</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+    <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" t="s">
-        <v>37</v>
-      </c>
-      <c r="D13" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14">
-        <v>2.0000000000000001E-4</v>
+        <v>11</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B15">
-        <v>0.03</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="C15" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D15" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B16">
-        <v>2.8500000000000001E-2</v>
+        <v>0.03</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B17">
-        <v>1.5E-3</v>
+        <v>2.8500000000000001E-2</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D17" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B18">
-        <v>1.6999999999999999E-3</v>
+        <v>1.5E-3</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D18" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B19">
-        <v>1E-4</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B20">
-        <v>0.95</v>
+        <v>1E-4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>54</v>
       </c>
       <c r="D20" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B21">
-        <v>0.05</v>
+        <v>0.95</v>
       </c>
       <c r="D21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B22">
-        <v>0.24912000000000001</v>
-      </c>
-      <c r="C22" t="s">
-        <v>61</v>
+        <v>0.05</v>
       </c>
       <c r="D22" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B23">
-        <v>4.7999999999999998E-6</v>
+        <v>0.24912000000000001</v>
       </c>
       <c r="C23" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B24">
-        <v>1.36E-5</v>
+        <v>4.7999999999999998E-6</v>
       </c>
       <c r="C24" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>66</v>
+      </c>
+      <c r="B25">
+        <v>1.36E-5</v>
+      </c>
+      <c r="C25" t="s">
+        <v>67</v>
+      </c>
+      <c r="D25" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>69</v>
       </c>
-      <c r="B25">
+      <c r="B26">
         <v>1000</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
+    <row r="28" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>11</v>
-      </c>
-      <c r="B28" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28" t="s">
-        <v>13</v>
-      </c>
-      <c r="D28" t="s">
-        <v>7</v>
-      </c>
-      <c r="E28" t="s">
-        <v>14</v>
-      </c>
-      <c r="F28" t="s">
-        <v>23</v>
-      </c>
-      <c r="G28" t="s">
-        <v>9</v>
-      </c>
-      <c r="H28" t="s">
-        <v>37</v>
-      </c>
-      <c r="I28" t="s">
-        <v>20</v>
-      </c>
-      <c r="J28" t="s">
-        <v>21</v>
-      </c>
-      <c r="K28" t="s">
-        <v>70</v>
-      </c>
-      <c r="L28" t="s">
-        <v>71</v>
-      </c>
-      <c r="M28" t="s">
-        <v>72</v>
-      </c>
-      <c r="N28" t="s">
-        <v>6</v>
-      </c>
-      <c r="O28" t="s">
-        <v>73</v>
-      </c>
-      <c r="P28" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>15</v>
-      </c>
-      <c r="R28" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>24</v>
-      </c>
-      <c r="B29">
-        <v>2.8499999999999998E-6</v>
+        <v>11</v>
+      </c>
+      <c r="B29" t="s">
+        <v>12</v>
       </c>
       <c r="C29" t="s">
-        <v>25</v>
+        <v>13</v>
+      </c>
+      <c r="D29" t="s">
+        <v>7</v>
       </c>
       <c r="E29" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F29" t="s">
-        <v>76</v>
+        <v>23</v>
       </c>
       <c r="G29" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="H29" t="s">
-        <v>77</v>
-      </c>
-      <c r="I29">
-        <v>2</v>
-      </c>
-      <c r="J29">
-        <v>-13.74250176111102</v>
-      </c>
-      <c r="K29">
-        <v>0.34942810419312298</v>
+        <v>37</v>
+      </c>
+      <c r="I29" t="s">
+        <v>20</v>
+      </c>
+      <c r="J29" t="s">
+        <v>21</v>
+      </c>
+      <c r="K29" t="s">
+        <v>70</v>
       </c>
       <c r="L29" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="M29" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="N29" t="s">
-        <v>132</v>
-      </c>
-      <c r="O29">
-        <v>2.8540000000000002E-3</v>
+        <v>6</v>
+      </c>
+      <c r="O29" t="s">
+        <v>73</v>
       </c>
       <c r="P29" t="s">
-        <v>80</v>
-      </c>
-      <c r="R29">
-        <v>0.2</v>
+        <v>74</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>15</v>
+      </c>
+      <c r="R29" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="B30">
-        <v>3.7367999999999999E-4</v>
+        <v>2.8499999999999998E-6</v>
       </c>
       <c r="C30" t="s">
         <v>25</v>
@@ -2008,42 +2963,42 @@
         <v>27</v>
       </c>
       <c r="H30" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="I30">
         <v>2</v>
       </c>
       <c r="J30">
-        <v>-4.781436711539472</v>
+        <v>-13.74250176111102</v>
       </c>
       <c r="K30">
-        <v>0.2046948949045872</v>
+        <v>0.34942810419312298</v>
       </c>
       <c r="L30" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="M30" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="N30" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O30">
-        <v>1.2659999999999999E-4</v>
+        <v>2.8540000000000002E-3</v>
       </c>
       <c r="P30" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="R30">
-        <v>2.4494897427831779E-2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>3.7367999999999999E-4</v>
       </c>
       <c r="C31" t="s">
         <v>25</v>
@@ -2057,34 +3012,43 @@
       <c r="G31" t="s">
         <v>27</v>
       </c>
+      <c r="H31" t="s">
+        <v>82</v>
+      </c>
       <c r="I31">
         <v>2</v>
       </c>
       <c r="J31">
-        <v>-11.84434628152367</v>
+        <v>-4.781436711539472</v>
       </c>
       <c r="K31">
-        <v>0.83144452611103292</v>
+        <v>0.2046948949045872</v>
       </c>
       <c r="L31" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="M31" t="s">
-        <v>88</v>
+        <v>84</v>
+      </c>
+      <c r="N31" t="s">
+        <v>133</v>
+      </c>
+      <c r="O31">
+        <v>1.2659999999999999E-4</v>
       </c>
       <c r="P31" t="s">
         <v>85</v>
       </c>
       <c r="R31">
-        <v>0.80622577482985502</v>
+        <v>2.4494897427831779E-2</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>86</v>
       </c>
       <c r="B32">
-        <v>2.0400000000000001E-8</v>
+        <v>0</v>
       </c>
       <c r="C32" t="s">
         <v>25</v>
@@ -2098,35 +3062,26 @@
       <c r="G32" t="s">
         <v>27</v>
       </c>
-      <c r="H32" t="s">
-        <v>89</v>
-      </c>
       <c r="I32">
         <v>2</v>
       </c>
       <c r="J32">
-        <v>-14.664736275474411</v>
+        <v>-11.84434628152367</v>
       </c>
       <c r="K32">
-        <v>0.2851315485876651</v>
+        <v>0.83144452611103292</v>
       </c>
       <c r="L32" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="M32" t="s">
-        <v>91</v>
-      </c>
-      <c r="N32" t="s">
-        <v>133</v>
-      </c>
-      <c r="O32">
-        <v>4.27746E-7</v>
+        <v>88</v>
       </c>
       <c r="P32" t="s">
         <v>85</v>
       </c>
       <c r="R32">
-        <v>0.2</v>
+        <v>0.80622577482985502</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.3">
@@ -2134,7 +3089,7 @@
         <v>28</v>
       </c>
       <c r="B33">
-        <v>5.6999999999999996E-6</v>
+        <v>2.0400000000000001E-8</v>
       </c>
       <c r="C33" t="s">
         <v>25</v>
@@ -2149,21 +3104,42 @@
         <v>27</v>
       </c>
       <c r="H33" t="s">
-        <v>92</v>
+        <v>89</v>
+      </c>
+      <c r="I33">
+        <v>2</v>
+      </c>
+      <c r="J33">
+        <v>-14.664736275474411</v>
+      </c>
+      <c r="K33">
+        <v>0.2851315485876651</v>
+      </c>
+      <c r="L33" t="s">
+        <v>90</v>
+      </c>
+      <c r="M33" t="s">
+        <v>91</v>
       </c>
       <c r="N33" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="O33">
-        <v>5.7000000000000002E-3</v>
+        <v>4.27746E-7</v>
+      </c>
+      <c r="P33" t="s">
+        <v>85</v>
+      </c>
+      <c r="R33">
+        <v>0.2</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>93</v>
+        <v>28</v>
       </c>
       <c r="B34">
-        <v>7.2E-9</v>
+        <v>5.6999999999999996E-6</v>
       </c>
       <c r="C34" t="s">
         <v>25</v>
@@ -2178,42 +3154,21 @@
         <v>27</v>
       </c>
       <c r="H34" t="s">
-        <v>94</v>
-      </c>
-      <c r="I34">
-        <v>2</v>
-      </c>
-      <c r="J34">
-        <v>-15.751988332064601</v>
-      </c>
-      <c r="K34">
-        <v>0.2851315485876651</v>
-      </c>
-      <c r="L34" t="s">
-        <v>95</v>
-      </c>
-      <c r="M34" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="N34" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="O34">
-        <v>1E-8</v>
-      </c>
-      <c r="P34" t="s">
-        <v>85</v>
-      </c>
-      <c r="R34">
-        <v>0.2</v>
+        <v>5.7000000000000002E-3</v>
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>29</v>
+        <v>93</v>
       </c>
       <c r="B35">
-        <v>0</v>
+        <v>7.2E-9</v>
       </c>
       <c r="C35" t="s">
         <v>25</v>
@@ -2227,13 +3182,43 @@
       <c r="G35" t="s">
         <v>27</v>
       </c>
+      <c r="H35" t="s">
+        <v>94</v>
+      </c>
+      <c r="I35">
+        <v>2</v>
+      </c>
+      <c r="J35">
+        <v>-15.751988332064601</v>
+      </c>
+      <c r="K35">
+        <v>0.2851315485876651</v>
+      </c>
+      <c r="L35" t="s">
+        <v>95</v>
+      </c>
+      <c r="M35" t="s">
+        <v>96</v>
+      </c>
+      <c r="N35" t="s">
+        <v>133</v>
+      </c>
+      <c r="O35">
+        <v>1E-8</v>
+      </c>
+      <c r="P35" t="s">
+        <v>85</v>
+      </c>
+      <c r="R35">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B36">
-        <v>4.8449999999999992E-5</v>
+        <v>0</v>
       </c>
       <c r="C36" t="s">
         <v>25</v>
@@ -2247,40 +3232,13 @@
       <c r="G36" t="s">
         <v>27</v>
       </c>
-      <c r="H36" t="s">
-        <v>97</v>
-      </c>
-      <c r="I36">
-        <v>2</v>
-      </c>
-      <c r="J36">
-        <v>-8.5295340272510369</v>
-      </c>
-      <c r="K36">
-        <v>0.2851315485876651</v>
-      </c>
-      <c r="M36" t="s">
-        <v>98</v>
-      </c>
-      <c r="N36" t="s">
-        <v>134</v>
-      </c>
-      <c r="O36">
-        <v>4.8512E-2</v>
-      </c>
-      <c r="P36" t="s">
-        <v>85</v>
-      </c>
-      <c r="R36">
-        <v>0.2</v>
-      </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B37">
-        <v>0</v>
+        <v>4.8449999999999992E-5</v>
       </c>
       <c r="C37" t="s">
         <v>25</v>
@@ -2294,25 +3252,37 @@
       <c r="G37" t="s">
         <v>27</v>
       </c>
+      <c r="H37" t="s">
+        <v>97</v>
+      </c>
       <c r="I37">
         <v>2</v>
       </c>
       <c r="J37">
-        <v>-12.26645129759965</v>
+        <v>-8.5295340272510369</v>
       </c>
       <c r="K37">
-        <v>0.58420886675914119</v>
+        <v>0.2851315485876651</v>
+      </c>
+      <c r="M37" t="s">
+        <v>98</v>
+      </c>
+      <c r="N37" t="s">
+        <v>134</v>
+      </c>
+      <c r="O37">
+        <v>4.8512E-2</v>
       </c>
       <c r="P37" t="s">
         <v>85</v>
       </c>
       <c r="R37">
-        <v>0.54772255750516607</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>99</v>
+        <v>31</v>
       </c>
       <c r="B38">
         <v>0</v>
@@ -2333,21 +3303,21 @@
         <v>2</v>
       </c>
       <c r="J38">
-        <v>-11.90977529142279</v>
+        <v>-12.26645129759965</v>
       </c>
       <c r="K38">
-        <v>0.40162171256046397</v>
+        <v>0.58420886675914119</v>
       </c>
       <c r="P38" t="s">
         <v>85</v>
       </c>
       <c r="R38">
-        <v>0.34641016151377552</v>
+        <v>0.54772255750516607</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -2368,21 +3338,21 @@
         <v>2</v>
       </c>
       <c r="J39">
-        <v>-12.132918842737</v>
+        <v>-11.90977529142279</v>
       </c>
       <c r="K39">
-        <v>0.58420886675914119</v>
+        <v>0.40162171256046397</v>
       </c>
       <c r="P39" t="s">
         <v>85</v>
       </c>
       <c r="R39">
-        <v>0.54772255750516607</v>
+        <v>0.34641016151377552</v>
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B40">
         <v>0</v>
@@ -2403,82 +3373,88 @@
         <v>2</v>
       </c>
       <c r="J40">
-        <v>-9.0081753390471704</v>
+        <v>-12.132918842737</v>
       </c>
       <c r="K40">
-        <v>0.2046948949045872</v>
-      </c>
-      <c r="L40" t="s">
-        <v>102</v>
-      </c>
-      <c r="M40" t="s">
-        <v>103</v>
+        <v>0.58420886675914119</v>
       </c>
       <c r="P40" t="s">
         <v>85</v>
       </c>
       <c r="R40">
-        <v>2.4494897427831779E-2</v>
+        <v>0.54772255750516607</v>
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>34</v>
+        <v>101</v>
       </c>
       <c r="B41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C41" t="s">
-        <v>125</v>
-      </c>
-      <c r="D41" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E41" t="s">
-        <v>16</v>
+        <v>26</v>
+      </c>
+      <c r="F41" t="s">
+        <v>76</v>
       </c>
       <c r="G41" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q41" t="s">
-        <v>19</v>
+        <v>27</v>
+      </c>
+      <c r="I41">
+        <v>2</v>
+      </c>
+      <c r="J41">
+        <v>-9.0081753390471704</v>
+      </c>
+      <c r="K41">
+        <v>0.2046948949045872</v>
+      </c>
+      <c r="L41" t="s">
+        <v>102</v>
+      </c>
+      <c r="M41" t="s">
+        <v>103</v>
+      </c>
+      <c r="P41" t="s">
+        <v>85</v>
+      </c>
+      <c r="R41">
+        <v>2.4494897427831779E-2</v>
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>139</v>
+        <v>34</v>
       </c>
       <c r="B42">
-        <v>2.8500000000000001E-2</v>
+        <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>22</v>
+        <v>125</v>
       </c>
       <c r="D42" t="s">
-        <v>104</v>
+        <v>8</v>
       </c>
       <c r="E42" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="G42" t="s">
-        <v>18</v>
-      </c>
-      <c r="H42" t="s">
-        <v>44</v>
-      </c>
-      <c r="O42">
-        <v>5.4999999999999997E-3</v>
+        <v>17</v>
       </c>
       <c r="Q42" t="s">
-        <v>105</v>
+        <v>19</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>106</v>
+        <v>139</v>
       </c>
       <c r="B43">
-        <v>-1.2999999999999999E-5</v>
+        <v>2.8500000000000001E-2</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
@@ -2492,40 +3468,28 @@
       <c r="G43" t="s">
         <v>18</v>
       </c>
-      <c r="I43">
-        <v>2</v>
-      </c>
-      <c r="J43">
-        <v>-11.61787681268815</v>
-      </c>
-      <c r="K43">
-        <v>0.21142374511865969</v>
-      </c>
-      <c r="N43" t="s">
-        <v>107</v>
-      </c>
-      <c r="P43" t="s">
-        <v>108</v>
+      <c r="H43" t="s">
+        <v>44</v>
+      </c>
+      <c r="O43">
+        <v>5.4999999999999997E-3</v>
       </c>
       <c r="Q43" t="s">
-        <v>109</v>
-      </c>
-      <c r="R43">
-        <v>2.4494897427831779E-2</v>
+        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B44">
-        <v>1.5E-3</v>
+        <v>-1.2999999999999999E-5</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E44" t="s">
         <v>26</v>
@@ -2533,63 +3497,63 @@
       <c r="G44" t="s">
         <v>18</v>
       </c>
-      <c r="H44" t="s">
-        <v>47</v>
-      </c>
-      <c r="O44">
-        <v>1.2659999999999999E-4</v>
+      <c r="I44">
+        <v>2</v>
+      </c>
+      <c r="J44">
+        <v>-11.61787681268815</v>
+      </c>
+      <c r="K44">
+        <v>0.21142374511865969</v>
+      </c>
+      <c r="N44" t="s">
+        <v>107</v>
+      </c>
+      <c r="P44" t="s">
+        <v>108</v>
       </c>
       <c r="Q44" t="s">
-        <v>112</v>
+        <v>109</v>
+      </c>
+      <c r="R44">
+        <v>2.4494897427831779E-2</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B45">
-        <v>1.0593999999999999E-11</v>
+        <v>1.5E-3</v>
       </c>
       <c r="C45" t="s">
         <v>22</v>
       </c>
       <c r="D45" t="s">
-        <v>8</v>
+        <v>111</v>
       </c>
       <c r="E45" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G45" t="s">
         <v>18</v>
       </c>
-      <c r="I45">
-        <v>2</v>
-      </c>
-      <c r="J45">
-        <v>-25.270733312806211</v>
-      </c>
-      <c r="K45">
-        <v>0.46540305112880392</v>
-      </c>
-      <c r="N45" t="s">
-        <v>114</v>
-      </c>
-      <c r="P45" t="s">
-        <v>115</v>
+      <c r="H45" t="s">
+        <v>47</v>
+      </c>
+      <c r="O45">
+        <v>1.2659999999999999E-4</v>
       </c>
       <c r="Q45" t="s">
-        <v>116</v>
-      </c>
-      <c r="R45">
-        <v>0.34641016151377552</v>
+        <v>112</v>
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>32</v>
+        <v>113</v>
       </c>
       <c r="B46">
-        <v>1.3798099999999999E-16</v>
+        <v>1.0593999999999999E-11</v>
       </c>
       <c r="C46" t="s">
         <v>22</v>
@@ -2607,30 +3571,30 @@
         <v>2</v>
       </c>
       <c r="J46">
-        <v>-36.519415679373957</v>
+        <v>-25.270733312806211</v>
       </c>
       <c r="K46">
-        <v>0.58702640485756685</v>
+        <v>0.46540305112880392</v>
       </c>
       <c r="N46" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="P46" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="Q46" t="s">
-        <v>33</v>
+        <v>116</v>
       </c>
       <c r="R46">
-        <v>0.54772255750516607</v>
+        <v>0.34641016151377552</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>119</v>
+        <v>32</v>
       </c>
       <c r="B47">
-        <v>1.0593999999999999E-11</v>
+        <v>1.3798099999999999E-16</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
@@ -2648,50 +3612,68 @@
         <v>2</v>
       </c>
       <c r="J47">
-        <v>-25.270733312806211</v>
+        <v>-36.519415679373957</v>
       </c>
       <c r="K47">
-        <v>0.46540305112880392</v>
+        <v>0.58702640485756685</v>
       </c>
       <c r="N47" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="P47" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="Q47" t="s">
-        <v>120</v>
+        <v>33</v>
       </c>
       <c r="R47">
-        <v>0.34641016151377552</v>
+        <v>0.54772255750516607</v>
       </c>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B48">
-        <v>0</v>
+        <v>1.0593999999999999E-11</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>104</v>
+        <v>8</v>
       </c>
       <c r="E48" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="G48" t="s">
         <v>18</v>
       </c>
+      <c r="I48">
+        <v>2</v>
+      </c>
+      <c r="J48">
+        <v>-25.270733312806211</v>
+      </c>
+      <c r="K48">
+        <v>0.46540305112880392</v>
+      </c>
+      <c r="N48" t="s">
+        <v>114</v>
+      </c>
+      <c r="P48" t="s">
+        <v>115</v>
+      </c>
       <c r="Q48" t="s">
-        <v>122</v>
+        <v>120</v>
+      </c>
+      <c r="R48">
+        <v>0.34641016151377552</v>
       </c>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B49">
         <v>0</v>
@@ -2709,6 +3691,29 @@
         <v>18</v>
       </c>
       <c r="Q49" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>123</v>
+      </c>
+      <c r="B50">
+        <v>0</v>
+      </c>
+      <c r="C50" t="s">
+        <v>22</v>
+      </c>
+      <c r="D50" t="s">
+        <v>104</v>
+      </c>
+      <c r="E50" t="s">
+        <v>26</v>
+      </c>
+      <c r="G50" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q50" t="s">
         <v>124</v>
       </c>
     </row>
@@ -2717,7 +3722,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6EFFFC2-89D0-45E5-B7FA-4B2E66075D0E}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
commenting for better understanding
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C8414FC-1405-4F9C-8A66-41FC458B3A88}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EDE1B97-7C35-432D-8D53-B8814D8B19BB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="174">
   <si>
     <t>Database</t>
   </si>
@@ -549,6 +549,21 @@
   </si>
   <si>
     <t>DE</t>
+  </si>
+  <si>
+    <t>market for transport, freight, lorry</t>
+  </si>
+  <si>
+    <t>transport, freight, lorry</t>
+  </si>
+  <si>
+    <t>transport, hydrogen, gaseous, lorry, unspecified</t>
+  </si>
+  <si>
+    <t>transport, hydrogen, liquid, lorry, unspecified</t>
+  </si>
+  <si>
+    <t>Hydrogen</t>
   </si>
 </sst>
 </file>
@@ -953,7 +968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="82.6640625" customWidth="1"/>
@@ -982,7 +997,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -1006,7 +1021,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -1067,7 +1082,7 @@
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="str">
         <f>B6</f>
-        <v>transport, hydrogen, gaseous, lorry, market average propulsion system</v>
+        <v>transport, hydrogen, gaseous, lorry, unspecified</v>
       </c>
       <c r="B12">
         <f>B5</f>
@@ -1084,7 +1099,7 @@
       </c>
       <c r="G12" t="str">
         <f>A12</f>
-        <v>transport, hydrogen, gaseous, lorry, market average propulsion system</v>
+        <v>transport, hydrogen, gaseous, lorry, unspecified</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -1115,8 +1130,8 @@
         <v>140</v>
       </c>
       <c r="B14">
-        <f>1*1000</f>
-        <v>1000</v>
+        <f>1*1000/540000</f>
+        <v>1.8518518518518519E-3</v>
       </c>
       <c r="C14" t="s">
         <v>8</v>
@@ -1158,203 +1173,197 @@
         <v>149</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>152</v>
-      </c>
-      <c r="B16">
+    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C16" t="s">
+        <v>165</v>
+      </c>
+      <c r="D16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17">
         <f>1000*0.005</f>
         <v>5</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D17" t="s">
         <v>26</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E17" t="s">
         <v>155</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F17" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+    <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>7</v>
-      </c>
-      <c r="B19" t="s">
-        <v>8</v>
+      <c r="B19" s="1" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>141</v>
-      </c>
-      <c r="B20">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B21" t="s">
-        <v>167</v>
+        <v>141</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>16</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>126</v>
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>6</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B25" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
+    <row r="26" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
         <v>11</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>12</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C27" t="s">
         <v>7</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D27" t="s">
         <v>14</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E27" t="s">
         <v>23</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F27" t="s">
         <v>9</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G27" t="s">
         <v>15</v>
       </c>
-      <c r="H26" t="s">
+      <c r="H27" t="s">
         <v>20</v>
       </c>
-      <c r="I26" t="s">
+      <c r="I27" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" t="str">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" t="str">
+        <f>B22</f>
+        <v>transport, hydrogen, liquid, lorry, unspecified</v>
+      </c>
+      <c r="B28">
         <f>B21</f>
-        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
-      </c>
-      <c r="B27">
-        <f>B20</f>
         <v>1</v>
       </c>
-      <c r="C27" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="C28" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" t="s">
         <v>16</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F28" t="s">
         <v>17</v>
       </c>
-      <c r="G27" t="str">
-        <f>A27</f>
-        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+      <c r="G28" t="str">
+        <f>A28</f>
+        <v>transport, hydrogen, liquid, lorry, unspecified</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>140</v>
       </c>
-      <c r="B28">
-        <v>1000</v>
-      </c>
-      <c r="C28" t="s">
-        <v>8</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="B29">
+        <f>1*1000/540000</f>
+        <v>1.8518518518518519E-3</v>
+      </c>
+      <c r="C29" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" t="s">
         <v>26</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F29" t="s">
         <v>18</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G29" t="s">
         <v>140</v>
       </c>
-      <c r="I28" t="s">
+      <c r="I29" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
+    <row r="30" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="B29">
+      <c r="B30">
         <f>1000*0.01625</f>
         <v>16.25</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C30" t="s">
         <v>165</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D30" t="s">
         <v>26</v>
-      </c>
-      <c r="F29" t="s">
-        <v>18</v>
-      </c>
-      <c r="G29" t="s">
-        <v>157</v>
-      </c>
-      <c r="I29" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>161</v>
-      </c>
-      <c r="B30">
-        <f>1000*6.78</f>
-        <v>6780</v>
-      </c>
-      <c r="C30" t="s">
-        <v>168</v>
-      </c>
-      <c r="D30" t="s">
-        <v>164</v>
       </c>
       <c r="F30" t="s">
         <v>18</v>
       </c>
       <c r="G30" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="I30" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
@@ -1362,7 +1371,8 @@
         <v>161</v>
       </c>
       <c r="B31">
-        <v>0.6</v>
+        <f>1000*6.78</f>
+        <v>6780</v>
       </c>
       <c r="C31" t="s">
         <v>168</v>
@@ -1377,166 +1387,170 @@
         <v>146</v>
       </c>
       <c r="I31" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="B32">
+        <f>1000*0.6</f>
+        <v>600</v>
+      </c>
+      <c r="C32" t="s">
+        <v>168</v>
+      </c>
+      <c r="D32" t="s">
+        <v>164</v>
+      </c>
+      <c r="F32" t="s">
+        <v>18</v>
+      </c>
+      <c r="G32" t="s">
+        <v>146</v>
+      </c>
+      <c r="I32" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>173</v>
+      </c>
+      <c r="B33">
         <f>1000*0.01625</f>
         <v>16.25</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D33" t="s">
         <v>26</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E33" t="s">
         <v>155</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F33" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+    <row r="35" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B35" s="1" t="s">
         <v>145</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>7</v>
-      </c>
-      <c r="B35" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>141</v>
-      </c>
-      <c r="B36">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="B36" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>15</v>
-      </c>
-      <c r="B37" t="s">
-        <v>145</v>
+        <v>141</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B38" t="s">
-        <v>16</v>
+        <v>145</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>126</v>
+        <v>14</v>
+      </c>
+      <c r="B39" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
         <v>6</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
+    <row r="42" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
         <v>11</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B43" t="s">
         <v>12</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C43" t="s">
         <v>7</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D43" t="s">
         <v>14</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E43" t="s">
         <v>23</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F43" t="s">
         <v>9</v>
       </c>
-      <c r="G42" t="s">
+      <c r="G43" t="s">
         <v>15</v>
       </c>
-      <c r="H42" t="s">
+      <c r="H43" t="s">
         <v>20</v>
       </c>
-      <c r="I42" t="s">
+      <c r="I43" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" t="str">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" t="str">
+        <f>B38</f>
+        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
+      </c>
+      <c r="B44">
         <f>B37</f>
-        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
-      </c>
-      <c r="B43">
-        <f>B36</f>
         <v>1</v>
       </c>
-      <c r="C43" t="s">
-        <v>8</v>
-      </c>
-      <c r="D43" t="s">
+      <c r="C44" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" t="s">
         <v>16</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F44" t="s">
         <v>17</v>
       </c>
-      <c r="G43" t="s">
+      <c r="G44" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
         <v>140</v>
       </c>
-      <c r="B44">
-        <f>1000*1</f>
-        <v>1000</v>
-      </c>
-      <c r="C44" t="s">
-        <v>8</v>
-      </c>
-      <c r="D44" t="s">
-        <v>26</v>
-      </c>
-      <c r="F44" t="s">
-        <v>18</v>
-      </c>
-      <c r="G44" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="4" t="s">
-        <v>156</v>
-      </c>
       <c r="B45">
-        <v>5.0000000000000001E-3</v>
+        <f>1000*1/540000</f>
+        <v>1.8518518518518519E-3</v>
       </c>
       <c r="C45" t="s">
-        <v>165</v>
+        <v>8</v>
       </c>
       <c r="D45" t="s">
         <v>26</v>
@@ -1545,167 +1559,167 @@
         <v>18</v>
       </c>
       <c r="G45" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>153</v>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>156</v>
       </c>
       <c r="B46">
-        <v>1</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="C46" t="s">
-        <v>8</v>
+        <v>165</v>
       </c>
       <c r="D46" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F46" t="s">
         <v>18</v>
       </c>
       <c r="G46" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>153</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" t="s">
+        <v>16</v>
+      </c>
+      <c r="F47" t="s">
+        <v>18</v>
+      </c>
+      <c r="G47" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="1" t="s">
+    <row r="49" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B49" s="1" t="s">
         <v>158</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>7</v>
-      </c>
-      <c r="B49" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>141</v>
-      </c>
-      <c r="B50">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="B50" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>15</v>
-      </c>
-      <c r="B51" t="s">
-        <v>158</v>
+        <v>141</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B52" t="s">
-        <v>16</v>
+        <v>158</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>126</v>
+        <v>14</v>
+      </c>
+      <c r="B53" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
         <v>6</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B55" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A55" s="1" t="s">
+    <row r="56" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>11</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B57" t="s">
         <v>12</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C57" t="s">
         <v>7</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D57" t="s">
         <v>14</v>
       </c>
-      <c r="E56" t="s">
+      <c r="E57" t="s">
         <v>23</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F57" t="s">
         <v>9</v>
       </c>
-      <c r="G56" t="s">
+      <c r="G57" t="s">
         <v>15</v>
       </c>
-      <c r="H56" t="s">
+      <c r="H57" t="s">
         <v>20</v>
       </c>
-      <c r="I56" t="s">
+      <c r="I57" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A57" t="str">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A58" t="str">
+        <f>B52</f>
+        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
+      </c>
+      <c r="B58">
         <f>B51</f>
-        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
-      </c>
-      <c r="B57">
-        <f>B50</f>
         <v>1</v>
       </c>
-      <c r="C57" t="s">
-        <v>8</v>
-      </c>
-      <c r="D57" t="s">
+      <c r="C58" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58" t="s">
         <v>16</v>
       </c>
-      <c r="F57" t="s">
+      <c r="F58" t="s">
         <v>17</v>
       </c>
-      <c r="G57" t="s">
+      <c r="G58" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
         <v>140</v>
       </c>
-      <c r="B58">
+      <c r="B59">
         <v>0</v>
       </c>
-      <c r="C58" t="s">
-        <v>8</v>
-      </c>
-      <c r="D58" t="s">
-        <v>26</v>
-      </c>
-      <c r="F58" t="s">
-        <v>18</v>
-      </c>
-      <c r="G58" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A59" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B59">
-        <v>5.0000000000000001E-3</v>
-      </c>
       <c r="C59" t="s">
-        <v>165</v>
+        <v>8</v>
       </c>
       <c r="D59" t="s">
         <v>26</v>
@@ -1714,38 +1728,55 @@
         <v>18</v>
       </c>
       <c r="G59" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>153</v>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A60" s="4" t="s">
+        <v>156</v>
       </c>
       <c r="B60">
-        <v>1</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="C60" t="s">
-        <v>8</v>
+        <v>165</v>
       </c>
       <c r="D60" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F60" t="s">
         <v>18</v>
       </c>
       <c r="G60" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>153</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61" t="s">
+        <v>16</v>
+      </c>
+      <c r="F61" t="s">
+        <v>18</v>
+      </c>
+      <c r="G61" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A62" s="1"/>
-      <c r="B62" s="1"/>
-    </row>
-    <row r="69" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A69" s="1"/>
-    </row>
-    <row r="72" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A72" s="4"/>
+    <row r="63" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A63" s="1"/>
+      <c r="B63" s="1"/>
+    </row>
+    <row r="70" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A70" s="1"/>
     </row>
     <row r="73" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A73" s="4"/>
@@ -1755,10 +1786,10 @@
     </row>
     <row r="75" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A75" s="4"/>
-      <c r="G75" s="4"/>
-    </row>
-    <row r="77" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A77" s="4"/>
+    </row>
+    <row r="76" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A76" s="4"/>
+      <c r="G76" s="4"/>
     </row>
     <row r="78" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A78" s="4"/>
@@ -1768,6 +1799,9 @@
     </row>
     <row r="80" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A80" s="4"/>
+    </row>
+    <row r="81" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A81" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>